<commit_message>
ci: production deploy tooling + GitHub Actions (build/e2e/publish GHCR)
- docker-compose.prod.yml: persistent storage volume + deterministic volume names
- docker-compose.e2e.yml: committed e2e stack (isolated postgis_e2e volume)
- docker-compose.yml: optional .env.local, default mysql password
- ci.yml: e2e (Playwright 27 tests) + publish image ke GHCR saat push main
- deploy/: cloudflared config/service/README (app.ravlyr.my.id), backup/restore scripts, SETUP-VPS.md runbook
</commit_message>
<xml_diff>
--- a/tests/e2e/fixtures/tanah-import-run.xlsx
+++ b/tests/e2e/fixtures/tanah-import-run.xlsx
@@ -417,7 +417,7 @@
         <v>1</v>
       </c>
       <c r="F7">
-        <v>940339</v>
+        <v>927730</v>
       </c>
       <c r="G7" t="s">
         <v>5</v>
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="F8">
-        <v>840339</v>
+        <v>827730</v>
       </c>
       <c r="G8" t="s">
         <v>7</v>
@@ -484,7 +484,7 @@
         <v>3</v>
       </c>
       <c r="F9">
-        <v>740339</v>
+        <v>727730</v>
       </c>
       <c r="G9" t="s">
         <v>5</v>

</xml_diff>

<commit_message>
fix: compose stack naming, e2e standalone (port 8081), prod port localhost-only, backup script container name
</commit_message>
<xml_diff>
--- a/tests/e2e/fixtures/tanah-import-run.xlsx
+++ b/tests/e2e/fixtures/tanah-import-run.xlsx
@@ -417,7 +417,7 @@
         <v>1</v>
       </c>
       <c r="F7">
-        <v>927730</v>
+        <v>939814</v>
       </c>
       <c r="G7" t="s">
         <v>5</v>
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="F8">
-        <v>827730</v>
+        <v>839814</v>
       </c>
       <c r="G8" t="s">
         <v>7</v>
@@ -484,7 +484,7 @@
         <v>3</v>
       </c>
       <c r="F9">
-        <v>727730</v>
+        <v>739814</v>
       </c>
       <c r="G9" t="s">
         <v>5</v>

</xml_diff>